<commit_message>
7-7 pc sport check
</commit_message>
<xml_diff>
--- a/delivery/final code/data/data partition-creative.xlsx
+++ b/delivery/final code/data/data partition-creative.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\R\Thesis\studies\AI ranking test\data for thesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\R\Thesis\Large-Choice-Sets-ranking\delivery\final code\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6262845-D07E-45BB-879C-253B2DBC87F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEFAC8FE-6E08-4D58-9764-52E8066B6440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E5A551B8-79B9-4C2C-9E1E-B1C876A2B4FE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E5A551B8-79B9-4C2C-9E1E-B1C876A2B4FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -721,9 +721,6 @@
 </t>
   </si>
   <si>
-    <t>Welcome to the future.  Upon entering this airport, you are greeted by one of several robots who are there to do initial check in.  These robots collect your information as well as all luggage to be checked in.  Your luggage is quickly dropped into one of several underground tunnels that meet your high-speed plane.  You are then escorted to one of two VIP waiting areas.  One is for work and the other for relaxation while you wait for plane departure. Your every need is taken care of here by humans.  The combination of AI and human interaction is the perfect balanced amount.</t>
-  </si>
-  <si>
     <t>the airport is filled with chatter and noise. you walk down the aisle way after check in and are greeted by a robot. here the robot asks if you have any questions about your upcoming travel destination. he then asks if you are hungry or thirsty. you say you would like a diet coke. you insert your card and out pops a diet coke, cold and crisp. so easy!  it makes you feel relaxed and at ease while you wait for your plane to arrive. when the plane arrives you are ushered off to board where more robots help put your luggage over head. then its time for takeoff!
 1. ride into the future
 2. super robot helper
@@ -996,12 +993,20 @@
 Part 1: Please write a story of an ideal experience a traveler might have in using this futuristic airport. The story should focus on what a traveler might see and experience in the airport, and how it will make them feel. This futuristic experience can be creative and does not need to be limited to today’s technologies; instead, focus on achieving your ideal experience. The story should be 100–200 words. 
 Part 2: Create three catchy marketing slogans that encapsulate the unique futuristic experiences mentioned in your story. Each of the three slogans should be within 2–10 words.</t>
   </si>
+  <si>
+    <t>Welcome to the future.  Upon entering this airport, you are greeted by one of several robots who are there to do initial check in.  
+These robots collect your information as well as all luggage to be checked in.  
+Your luggage is quickly dropped into one of several underground tunnels that meet your high-speed plane.  
+You are then escorted to one of two VIP waiting areas.  
+One is for work and the other for relaxation while you wait for plane departure. Your every need is taken care of here by humans.  The combination of AI and human interaction is the perfect balanced amount.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1012,6 +1017,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="136"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1035,10 +1048,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1257,12 +1273,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C2D6F55-D426-4F56-9227-4290A18ED1B4}">
   <dimension ref="A1:B160"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="71.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -1270,7 +1287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>2</v>
       </c>
@@ -1278,7 +1295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>3</v>
       </c>
@@ -1286,7 +1303,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>4</v>
       </c>
@@ -1294,7 +1311,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>5</v>
       </c>
@@ -1302,7 +1319,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>6</v>
       </c>
@@ -1310,7 +1327,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>7</v>
       </c>
@@ -1318,7 +1335,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>8</v>
       </c>
@@ -1326,7 +1343,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>9</v>
       </c>
@@ -1334,7 +1351,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>10</v>
       </c>
@@ -1342,7 +1359,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>11</v>
       </c>
@@ -1350,7 +1367,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>12</v>
       </c>
@@ -1358,7 +1375,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>13</v>
       </c>
@@ -1366,7 +1383,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>14</v>
       </c>
@@ -1374,7 +1391,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>15</v>
       </c>
@@ -1382,7 +1399,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>16</v>
       </c>
@@ -1390,7 +1407,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>17</v>
       </c>
@@ -1398,7 +1415,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>18</v>
       </c>
@@ -1406,7 +1423,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>19</v>
       </c>
@@ -1414,7 +1431,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>20</v>
       </c>
@@ -1422,7 +1439,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>21</v>
       </c>
@@ -1430,7 +1447,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>22</v>
       </c>
@@ -1438,7 +1455,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>23</v>
       </c>
@@ -1446,7 +1463,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>24</v>
       </c>
@@ -1454,7 +1471,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>25</v>
       </c>
@@ -1462,7 +1479,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>26</v>
       </c>
@@ -1470,7 +1487,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>27</v>
       </c>
@@ -1478,7 +1495,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>28</v>
       </c>
@@ -1486,7 +1503,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>29</v>
       </c>
@@ -1494,7 +1511,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>30</v>
       </c>
@@ -1502,7 +1519,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>31</v>
       </c>
@@ -1510,7 +1527,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>32</v>
       </c>
@@ -1518,7 +1535,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>33</v>
       </c>
@@ -1526,7 +1543,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>34</v>
       </c>
@@ -1534,7 +1551,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>35</v>
       </c>
@@ -1542,7 +1559,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>36</v>
       </c>
@@ -1550,7 +1567,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>37</v>
       </c>
@@ -1558,7 +1575,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>38</v>
       </c>
@@ -1566,7 +1583,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>39</v>
       </c>
@@ -1574,7 +1591,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>40</v>
       </c>
@@ -1582,7 +1599,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>41</v>
       </c>
@@ -1590,7 +1607,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>42</v>
       </c>
@@ -1598,7 +1615,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>43</v>
       </c>
@@ -1606,7 +1623,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>44</v>
       </c>
@@ -1614,7 +1631,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>45</v>
       </c>
@@ -1622,7 +1639,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>46</v>
       </c>
@@ -1630,7 +1647,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>47</v>
       </c>
@@ -1638,7 +1655,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>48</v>
       </c>
@@ -1646,7 +1663,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>49</v>
       </c>
@@ -1654,7 +1671,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>50</v>
       </c>
@@ -1662,7 +1679,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>51</v>
       </c>
@@ -1670,7 +1687,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>52</v>
       </c>
@@ -1678,7 +1695,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>53</v>
       </c>
@@ -1686,7 +1703,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>54</v>
       </c>
@@ -1694,7 +1711,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>55</v>
       </c>
@@ -1702,7 +1719,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>56</v>
       </c>
@@ -1710,7 +1727,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>57</v>
       </c>
@@ -1718,7 +1735,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>58</v>
       </c>
@@ -1726,7 +1743,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>59</v>
       </c>
@@ -1734,7 +1751,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>60</v>
       </c>
@@ -1742,7 +1759,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>61</v>
       </c>
@@ -1750,7 +1767,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>62</v>
       </c>
@@ -1758,7 +1775,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>63</v>
       </c>
@@ -1766,7 +1783,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>64</v>
       </c>
@@ -1774,7 +1791,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>65</v>
       </c>
@@ -1782,7 +1799,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>66</v>
       </c>
@@ -1790,7 +1807,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>67</v>
       </c>
@@ -1798,7 +1815,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>68</v>
       </c>
@@ -1806,7 +1823,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>69</v>
       </c>
@@ -1814,7 +1831,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>70</v>
       </c>
@@ -1822,7 +1839,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>71</v>
       </c>
@@ -1830,7 +1847,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>72</v>
       </c>
@@ -1838,7 +1855,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>73</v>
       </c>
@@ -1846,7 +1863,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>74</v>
       </c>
@@ -1854,7 +1871,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>75</v>
       </c>
@@ -1862,7 +1879,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>76</v>
       </c>
@@ -1870,7 +1887,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>77</v>
       </c>
@@ -1878,7 +1895,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>78</v>
       </c>
@@ -1886,7 +1903,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>79</v>
       </c>
@@ -1894,7 +1911,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>80</v>
       </c>
@@ -1902,7 +1919,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>81</v>
       </c>
@@ -1910,7 +1927,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>82</v>
       </c>
@@ -1918,7 +1935,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
         <v>83</v>
       </c>
@@ -1926,7 +1943,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
         <v>84</v>
       </c>
@@ -1934,7 +1951,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
         <v>85</v>
       </c>
@@ -1942,7 +1959,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
         <v>86</v>
       </c>
@@ -1950,7 +1967,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
         <v>87</v>
       </c>
@@ -1958,7 +1975,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
         <v>88</v>
       </c>
@@ -1966,7 +1983,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>89</v>
       </c>
@@ -1974,7 +1991,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>90</v>
       </c>
@@ -1982,7 +1999,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>91</v>
       </c>
@@ -1990,7 +2007,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>92</v>
       </c>
@@ -1998,7 +2015,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>93</v>
       </c>
@@ -2006,7 +2023,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>94</v>
       </c>
@@ -2014,7 +2031,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
         <v>95</v>
       </c>
@@ -2022,7 +2039,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
         <v>96</v>
       </c>
@@ -2030,7 +2047,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
         <v>97</v>
       </c>
@@ -2038,7 +2055,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
         <v>98</v>
       </c>
@@ -2046,7 +2063,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
         <v>99</v>
       </c>
@@ -2054,7 +2071,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
         <v>100</v>
       </c>
@@ -2062,7 +2079,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" s="1">
         <v>101</v>
       </c>
@@ -2070,7 +2087,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" s="1">
         <v>102</v>
       </c>
@@ -2078,7 +2095,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" s="1">
         <v>103</v>
       </c>
@@ -2086,7 +2103,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" s="1">
         <v>104</v>
       </c>
@@ -2094,7 +2111,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" s="1">
         <v>105</v>
       </c>
@@ -2102,7 +2119,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" s="1">
         <v>106</v>
       </c>
@@ -2110,7 +2127,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" s="1">
         <v>107</v>
       </c>
@@ -2118,7 +2135,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" s="1">
         <v>108</v>
       </c>
@@ -2126,7 +2143,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" s="1">
         <v>109</v>
       </c>
@@ -2134,415 +2151,416 @@
         <v>108</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" ht="255" x14ac:dyDescent="0.2">
       <c r="A110" s="1">
         <v>110</v>
       </c>
-      <c r="B110" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B110" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" s="1">
         <v>111</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A112" s="1">
         <v>112</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A113" s="1">
         <v>113</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A114" s="1">
         <v>114</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A115" s="1">
         <v>115</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A116" s="1">
         <v>116</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" s="1">
         <v>117</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" s="1">
         <v>118</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" s="1">
         <v>119</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" s="1">
         <v>120</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" s="1">
         <v>121</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" s="1">
         <v>122</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" s="1">
         <v>123</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" s="1">
         <v>124</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A125" s="1">
         <v>125</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A126" s="1">
         <v>126</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A127" s="1">
         <v>127</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" s="1">
         <v>128</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" s="1">
         <v>129</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" s="1">
         <v>130</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A131" s="1">
         <v>131</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A132" s="1">
         <v>132</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A133" s="1">
         <v>133</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A134" s="1">
         <v>134</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" s="1">
         <v>135</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" s="1">
         <v>136</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" s="1">
         <v>137</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" s="1">
         <v>138</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" s="1">
         <v>139</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A140" s="1">
         <v>140</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A141" s="1">
         <v>141</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A142" s="1">
         <v>142</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A143" s="1">
         <v>143</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A144" s="1">
         <v>144</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A145" s="1">
         <v>145</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A146" s="1">
         <v>146</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A147" s="1">
         <v>147</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A148" s="1">
         <v>148</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A149" s="1">
         <v>149</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A150" s="1">
         <v>150</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A151" s="1">
         <v>151</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A152" s="1">
         <v>152</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A153" s="1">
         <v>153</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A154" s="1">
         <v>154</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A155" s="1">
         <v>155</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A156" s="1">
         <v>156</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A157" s="1">
         <v>157</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A158" s="1">
         <v>158</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A159" s="1">
         <v>159</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A160" s="1">
         <v>160</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2550,15 +2568,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C122B07E-2CB9-4E10-A4A4-CDDDEA7F391C}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="409.6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B1" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>